<commit_message>
Kész a címzés a szerverre
</commit_message>
<xml_diff>
--- a/Network/02.09 cimzes.xlsx
+++ b/Network/02.09 cimzes.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Github Repo\final-project-2025-26\Network\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Felhasználó.GEP.000\Desktop\Vizsgaremek\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D59BFEF3-6B4F-459B-8470-C425905C2F82}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{605007E4-4426-4662-9E25-34E4754AFAF4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-105" windowWidth="29040" windowHeight="15840" activeTab="3" xr2:uid="{6F35F872-ABCC-42C2-B031-C1DE53122CDE}"/>
   </bookViews>
@@ -17,18 +17,28 @@
     <sheet name="Fix IPk" sheetId="2" r:id="rId2"/>
     <sheet name="ISP Full Mesh" sheetId="4" r:id="rId3"/>
     <sheet name="OceanData" sheetId="3" r:id="rId4"/>
+    <sheet name="szerverek" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="427" uniqueCount="188">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="497" uniqueCount="229">
   <si>
     <t>Név</t>
   </si>
@@ -459,42 +469,6 @@
     <t>AD DNS</t>
   </si>
   <si>
-    <t>SQL</t>
-  </si>
-  <si>
-    <t>Fa0</t>
-  </si>
-  <si>
-    <t>Fa1</t>
-  </si>
-  <si>
-    <t>Linux FTP</t>
-  </si>
-  <si>
-    <t>SQL BACKUP</t>
-  </si>
-  <si>
-    <t>BACKUP SERVER1</t>
-  </si>
-  <si>
-    <t>LS1</t>
-  </si>
-  <si>
-    <t>LS2</t>
-  </si>
-  <si>
-    <t>LS3</t>
-  </si>
-  <si>
-    <t>LS4</t>
-  </si>
-  <si>
-    <t>LS5</t>
-  </si>
-  <si>
-    <t>Fa0/1</t>
-  </si>
-  <si>
     <t>Fa0/2</t>
   </si>
   <si>
@@ -516,82 +490,241 @@
     <t>MLS3</t>
   </si>
   <si>
+    <t>192.168.20.2</t>
+  </si>
+  <si>
+    <t>MLS4</t>
+  </si>
+  <si>
+    <t>AD DNS FRI</t>
+  </si>
+  <si>
+    <t>AD DNS BKP</t>
+  </si>
+  <si>
+    <t>FS</t>
+  </si>
+  <si>
+    <t>SQL PRI</t>
+  </si>
+  <si>
+    <t>SQL BKP</t>
+  </si>
+  <si>
+    <t>LINUX DB</t>
+  </si>
+  <si>
+    <t>LINUX WEB CRON CUPS</t>
+  </si>
+  <si>
+    <t>192.168.20.6</t>
+  </si>
+  <si>
+    <t>192.168.20.22</t>
+  </si>
+  <si>
+    <t>192.168.20.38</t>
+  </si>
+  <si>
+    <t>192.168.20.54</t>
+  </si>
+  <si>
+    <t>192.168.20.70</t>
+  </si>
+  <si>
+    <t>192.168.20.86</t>
+  </si>
+  <si>
+    <t>192.168.20.102</t>
+  </si>
+  <si>
+    <t>192.168.10.0/30</t>
+  </si>
+  <si>
+    <t>192.168.20.0/30</t>
+  </si>
+  <si>
+    <t>192.168.30.0/30</t>
+  </si>
+  <si>
+    <t>192.168.40.0/30</t>
+  </si>
+  <si>
+    <t>192.168.50.0/30</t>
+  </si>
+  <si>
+    <t>192.168.60.0/30</t>
+  </si>
+  <si>
+    <t>192.168.70.0/30</t>
+  </si>
+  <si>
+    <t>MLS5</t>
+  </si>
+  <si>
+    <t>MLS6</t>
+  </si>
+  <si>
+    <t>MLS7</t>
+  </si>
+  <si>
+    <t>VLAN10</t>
+  </si>
+  <si>
+    <t>VLAN20</t>
+  </si>
+  <si>
+    <t>VLAN30</t>
+  </si>
+  <si>
+    <t>VLAN40</t>
+  </si>
+  <si>
+    <t>VLAN50</t>
+  </si>
+  <si>
+    <t>VLAN60</t>
+  </si>
+  <si>
+    <t>VLAN70</t>
+  </si>
+  <si>
+    <t>SR1</t>
+  </si>
+  <si>
+    <t>Fa0/0</t>
+  </si>
+  <si>
+    <t>Fa1/0</t>
+  </si>
+  <si>
     <t>192.168.10.2</t>
   </si>
   <si>
-    <t>192.168.10.3</t>
-  </si>
-  <si>
-    <t>192.168.10.4</t>
-  </si>
-  <si>
-    <t>192.168.10.5</t>
-  </si>
-  <si>
-    <t>192.168.10.6</t>
-  </si>
-  <si>
-    <t>192.168.10.7</t>
-  </si>
-  <si>
-    <t>192.168.10.8</t>
-  </si>
-  <si>
-    <t>192.168.10.9</t>
-  </si>
-  <si>
-    <t>192.168.10.10</t>
-  </si>
-  <si>
-    <t>192.168.10.11</t>
-  </si>
-  <si>
-    <t>192.168.10.12</t>
-  </si>
-  <si>
-    <t>192.168.10.13</t>
-  </si>
-  <si>
-    <t>192.168.10.14</t>
-  </si>
-  <si>
-    <t>192.168.10.15</t>
-  </si>
-  <si>
-    <t>192.168.10.16</t>
-  </si>
-  <si>
-    <t>HSRP route: 192.168.10.1</t>
-  </si>
-  <si>
-    <t>192.168.10.20</t>
-  </si>
-  <si>
-    <t>192.168.10.21</t>
-  </si>
-  <si>
-    <t>192.168.10.22</t>
-  </si>
-  <si>
-    <t>192.168.10.23</t>
-  </si>
-  <si>
-    <t>192.168.10.24</t>
-  </si>
-  <si>
-    <t>192.168.10.25</t>
-  </si>
-  <si>
-    <t>192.168.10.26</t>
-  </si>
-  <si>
-    <t>192.168.10.27</t>
-  </si>
-  <si>
-    <t>192.168.10.28</t>
-  </si>
-  <si>
-    <t>192.168.10.29</t>
+    <t>192.168.30.2</t>
+  </si>
+  <si>
+    <t>192.168.40.2</t>
+  </si>
+  <si>
+    <t>192.168.50.2</t>
+  </si>
+  <si>
+    <t>192.168.60.2</t>
+  </si>
+  <si>
+    <t>192.168.70.2</t>
+  </si>
+  <si>
+    <t>SR2</t>
+  </si>
+  <si>
+    <t>Fa2/0</t>
+  </si>
+  <si>
+    <t>Fa3/0</t>
+  </si>
+  <si>
+    <t>Fa4/0</t>
+  </si>
+  <si>
+    <t>Fa5/0</t>
+  </si>
+  <si>
+    <t>Fa6/0</t>
+  </si>
+  <si>
+    <t>SR3</t>
+  </si>
+  <si>
+    <t>SR4</t>
+  </si>
+  <si>
+    <t>1.1.1.0</t>
+  </si>
+  <si>
+    <t>2.2.2.0</t>
+  </si>
+  <si>
+    <t>3.3.3.0</t>
+  </si>
+  <si>
+    <t>4.4.4.0</t>
+  </si>
+  <si>
+    <t>1.1.2.0</t>
+  </si>
+  <si>
+    <t>1.1.3.0</t>
+  </si>
+  <si>
+    <t>1.1.4.0</t>
+  </si>
+  <si>
+    <t>1.1.5.0</t>
+  </si>
+  <si>
+    <t>1.1.6.0</t>
+  </si>
+  <si>
+    <t>1.1.7.0</t>
+  </si>
+  <si>
+    <t>2.2.1.0</t>
+  </si>
+  <si>
+    <t>2.2.3.0</t>
+  </si>
+  <si>
+    <t>2.2.4.0</t>
+  </si>
+  <si>
+    <t>2.2.5.0</t>
+  </si>
+  <si>
+    <t>2.2.6.0</t>
+  </si>
+  <si>
+    <t>2.2.7.0</t>
+  </si>
+  <si>
+    <t>3.3.1.0</t>
+  </si>
+  <si>
+    <t>3.3.2.0</t>
+  </si>
+  <si>
+    <t>3.3.4.0</t>
+  </si>
+  <si>
+    <t>3.3.5.0</t>
+  </si>
+  <si>
+    <t>3.3.6.0</t>
+  </si>
+  <si>
+    <t>3.3.7.0</t>
+  </si>
+  <si>
+    <t>4.4.1.0</t>
+  </si>
+  <si>
+    <t>4.4.2.0</t>
+  </si>
+  <si>
+    <t>4.4.3.0</t>
+  </si>
+  <si>
+    <t>4.4.5.0</t>
+  </si>
+  <si>
+    <t>4.4.6.0</t>
+  </si>
+  <si>
+    <t>4.4.7.0</t>
+  </si>
+  <si>
+    <t>AD DNS PRI</t>
   </si>
 </sst>
 </file>
@@ -631,7 +764,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="17">
+  <fills count="16">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -718,12 +851,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.79998168889431442"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="2" tint="-9.9978637043366805E-2"/>
         <bgColor indexed="64"/>
       </patternFill>
@@ -765,7 +892,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
@@ -805,17 +932,9 @@
     <xf numFmtId="0" fontId="0" fillId="13" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="14" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
+    <xf numFmtId="2" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="0" fillId="10" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="15" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="15" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="16" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="16" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normál" xfId="0" builtinId="0"/>
@@ -2236,454 +2355,696 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D1D6D1D5-74AF-4AB6-A0A1-6D17E92BA017}">
-  <dimension ref="A2:G28"/>
+  <dimension ref="A2:J30"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="16.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="21.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.85546875" customWidth="1"/>
     <col min="3" max="3" width="17.7109375" customWidth="1"/>
     <col min="4" max="4" width="18.85546875" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="19.140625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="23" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="19" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A2" s="14"/>
-      <c r="B2" s="14"/>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>228</v>
+      </c>
+      <c r="B2" s="14" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>153</v>
+      </c>
+      <c r="B3" s="14" t="s">
+        <v>150</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>183</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>184</v>
+      </c>
+      <c r="H3" s="3" t="s">
+        <v>147</v>
+      </c>
+      <c r="I3" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="J3" s="25" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>154</v>
+      </c>
+      <c r="B4" s="14" t="s">
+        <v>187</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>183</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="H4" s="3" t="s">
+        <v>148</v>
+      </c>
+      <c r="I4" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="J4" s="3" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>155</v>
+      </c>
+      <c r="B5" s="14" t="s">
+        <v>188</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>183</v>
+      </c>
+      <c r="G5" s="3" t="s">
+        <v>193</v>
+      </c>
+      <c r="H5" s="3" t="s">
+        <v>149</v>
+      </c>
+      <c r="I5" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="J5" s="3" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>156</v>
+      </c>
+      <c r="B6" s="14" t="s">
+        <v>189</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>183</v>
+      </c>
+      <c r="G6" s="3" t="s">
+        <v>194</v>
+      </c>
+      <c r="H6" s="3" t="s">
+        <v>151</v>
+      </c>
+      <c r="I6" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="J6" s="25" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>157</v>
+      </c>
+      <c r="B7" s="14" t="s">
+        <v>190</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>183</v>
+      </c>
+      <c r="G7" s="3" t="s">
+        <v>195</v>
+      </c>
+      <c r="H7" s="3" t="s">
+        <v>173</v>
+      </c>
+      <c r="I7" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="J7" s="3" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>158</v>
+      </c>
+      <c r="B8" s="14" t="s">
+        <v>191</v>
+      </c>
+      <c r="F8" s="3" t="s">
+        <v>183</v>
+      </c>
+      <c r="G8" s="3" t="s">
+        <v>196</v>
+      </c>
+      <c r="H8" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="I8" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="J8" s="3" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="B9" s="14"/>
+      <c r="F9" s="3" t="s">
+        <v>183</v>
+      </c>
+      <c r="G9" s="3" t="s">
+        <v>197</v>
+      </c>
+      <c r="H9" s="3" t="s">
+        <v>175</v>
+      </c>
+      <c r="I9" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="J9" s="25" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="B10" s="14"/>
+      <c r="F10" s="19" t="s">
+        <v>192</v>
+      </c>
+      <c r="G10" s="19" t="s">
+        <v>184</v>
+      </c>
+      <c r="H10" s="19" t="s">
+        <v>147</v>
+      </c>
+      <c r="I10" s="19" t="s">
+        <v>144</v>
+      </c>
+      <c r="J10" s="26" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
         <v>142</v>
       </c>
-      <c r="B3" s="14" t="s">
+      <c r="B11" s="14" t="s">
+        <v>166</v>
+      </c>
+      <c r="C11" t="s">
+        <v>176</v>
+      </c>
+      <c r="D11" t="s">
+        <v>147</v>
+      </c>
+      <c r="F11" s="19" t="s">
+        <v>192</v>
+      </c>
+      <c r="G11" s="19" t="s">
+        <v>185</v>
+      </c>
+      <c r="H11" s="19" t="s">
+        <v>148</v>
+      </c>
+      <c r="I11" s="19" t="s">
         <v>144</v>
       </c>
-      <c r="C3" t="s">
+      <c r="J11" s="19" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>153</v>
+      </c>
+      <c r="B12" s="14" t="s">
+        <v>167</v>
+      </c>
+      <c r="C12" t="s">
+        <v>177</v>
+      </c>
+      <c r="D12" t="s">
+        <v>148</v>
+      </c>
+      <c r="F12" s="19" t="s">
+        <v>192</v>
+      </c>
+      <c r="G12" s="19" t="s">
+        <v>193</v>
+      </c>
+      <c r="H12" s="19" t="s">
+        <v>149</v>
+      </c>
+      <c r="I12" s="19" t="s">
+        <v>144</v>
+      </c>
+      <c r="J12" s="19" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>154</v>
+      </c>
+      <c r="B13" s="14" t="s">
+        <v>168</v>
+      </c>
+      <c r="C13" t="s">
         <v>178</v>
       </c>
-      <c r="D3" t="s">
+      <c r="D13" t="s">
         <v>149</v>
       </c>
-      <c r="E3" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>142</v>
-      </c>
-      <c r="B4" s="14" t="s">
+      <c r="F13" s="19" t="s">
+        <v>192</v>
+      </c>
+      <c r="G13" s="19" t="s">
+        <v>194</v>
+      </c>
+      <c r="H13" s="19" t="s">
+        <v>151</v>
+      </c>
+      <c r="I13" s="19" t="s">
+        <v>144</v>
+      </c>
+      <c r="J13" s="19" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>155</v>
+      </c>
+      <c r="B14" s="14" t="s">
+        <v>169</v>
+      </c>
+      <c r="C14" t="s">
+        <v>179</v>
+      </c>
+      <c r="D14" t="s">
+        <v>151</v>
+      </c>
+      <c r="F14" s="19" t="s">
+        <v>192</v>
+      </c>
+      <c r="G14" s="19" t="s">
+        <v>195</v>
+      </c>
+      <c r="H14" s="19" t="s">
+        <v>173</v>
+      </c>
+      <c r="I14" s="19" t="s">
+        <v>144</v>
+      </c>
+      <c r="J14" s="19" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>156</v>
+      </c>
+      <c r="B15" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="C15" t="s">
+        <v>180</v>
+      </c>
+      <c r="D15" t="s">
+        <v>173</v>
+      </c>
+      <c r="F15" s="19" t="s">
+        <v>192</v>
+      </c>
+      <c r="G15" s="19" t="s">
+        <v>196</v>
+      </c>
+      <c r="H15" s="19" t="s">
+        <v>174</v>
+      </c>
+      <c r="I15" s="19" t="s">
+        <v>144</v>
+      </c>
+      <c r="J15" s="19" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>157</v>
+      </c>
+      <c r="B16" s="14" t="s">
+        <v>171</v>
+      </c>
+      <c r="C16" t="s">
+        <v>181</v>
+      </c>
+      <c r="D16" t="s">
+        <v>174</v>
+      </c>
+      <c r="F16" s="19" t="s">
+        <v>192</v>
+      </c>
+      <c r="G16" s="19" t="s">
+        <v>197</v>
+      </c>
+      <c r="H16" s="19" t="s">
+        <v>175</v>
+      </c>
+      <c r="I16" s="19" t="s">
+        <v>144</v>
+      </c>
+      <c r="J16" s="19" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>158</v>
+      </c>
+      <c r="B17" s="14" t="s">
+        <v>172</v>
+      </c>
+      <c r="C17" t="s">
+        <v>182</v>
+      </c>
+      <c r="D17" t="s">
+        <v>175</v>
+      </c>
+      <c r="F17" s="27" t="s">
+        <v>198</v>
+      </c>
+      <c r="G17" s="27" t="s">
+        <v>184</v>
+      </c>
+      <c r="H17" s="27" t="s">
+        <v>147</v>
+      </c>
+      <c r="I17" s="27" t="s">
         <v>145</v>
       </c>
-      <c r="C4" t="s">
-        <v>179</v>
-      </c>
-      <c r="D4" t="s">
+      <c r="J17" s="27" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="F18" s="27" t="s">
+        <v>198</v>
+      </c>
+      <c r="G18" s="27" t="s">
+        <v>185</v>
+      </c>
+      <c r="H18" s="27" t="s">
+        <v>148</v>
+      </c>
+      <c r="I18" s="27" t="s">
+        <v>145</v>
+      </c>
+      <c r="J18" s="27" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="F19" s="27" t="s">
+        <v>198</v>
+      </c>
+      <c r="G19" s="27" t="s">
+        <v>193</v>
+      </c>
+      <c r="H19" s="27" t="s">
         <v>149</v>
       </c>
-      <c r="E4" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>143</v>
-      </c>
-      <c r="B5" s="14" t="s">
-        <v>144</v>
-      </c>
-      <c r="C5" t="s">
-        <v>180</v>
-      </c>
-      <c r="D5" t="s">
-        <v>150</v>
-      </c>
-      <c r="E5" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>143</v>
-      </c>
-      <c r="B6" s="14" t="s">
+      <c r="I19" s="27" t="s">
         <v>145</v>
       </c>
-      <c r="C6" t="s">
-        <v>181</v>
-      </c>
-      <c r="D6" t="s">
-        <v>150</v>
-      </c>
-      <c r="E6" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
+      <c r="J19" s="27" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="F20" s="27" t="s">
+        <v>198</v>
+      </c>
+      <c r="G20" s="27" t="s">
+        <v>194</v>
+      </c>
+      <c r="H20" s="27" t="s">
+        <v>151</v>
+      </c>
+      <c r="I20" s="27" t="s">
+        <v>145</v>
+      </c>
+      <c r="J20" s="27" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="F21" s="27" t="s">
+        <v>198</v>
+      </c>
+      <c r="G21" s="27" t="s">
+        <v>195</v>
+      </c>
+      <c r="H21" s="27" t="s">
+        <v>173</v>
+      </c>
+      <c r="I21" s="27" t="s">
+        <v>145</v>
+      </c>
+      <c r="J21" s="27" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="F22" s="27" t="s">
+        <v>198</v>
+      </c>
+      <c r="G22" s="27" t="s">
+        <v>196</v>
+      </c>
+      <c r="H22" s="27" t="s">
+        <v>174</v>
+      </c>
+      <c r="I22" s="27" t="s">
+        <v>145</v>
+      </c>
+      <c r="J22" s="27" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="F23" s="27" t="s">
+        <v>198</v>
+      </c>
+      <c r="G23" s="27" t="s">
+        <v>197</v>
+      </c>
+      <c r="H23" s="27" t="s">
+        <v>175</v>
+      </c>
+      <c r="I23" s="27" t="s">
+        <v>145</v>
+      </c>
+      <c r="J23" s="27" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="24" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="F24" s="2" t="s">
+        <v>199</v>
+      </c>
+      <c r="G24" s="2" t="s">
+        <v>184</v>
+      </c>
+      <c r="H24" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="I24" s="2" t="s">
         <v>146</v>
       </c>
-      <c r="B7" s="14" t="s">
-        <v>144</v>
-      </c>
-      <c r="C7" t="s">
-        <v>182</v>
-      </c>
-      <c r="D7" t="s">
+      <c r="J24" s="2" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="F25" s="2" t="s">
+        <v>199</v>
+      </c>
+      <c r="G25" s="2" t="s">
+        <v>185</v>
+      </c>
+      <c r="H25" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="I25" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="J25" s="2" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="F26" s="2" t="s">
+        <v>199</v>
+      </c>
+      <c r="G26" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="H26" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="I26" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="J26" s="2" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="27" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="F27" s="2" t="s">
+        <v>199</v>
+      </c>
+      <c r="G27" s="2" t="s">
+        <v>194</v>
+      </c>
+      <c r="H27" s="2" t="s">
         <v>151</v>
       </c>
-      <c r="E7" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
+      <c r="I27" s="2" t="s">
         <v>146</v>
       </c>
-      <c r="B8" s="14" t="s">
-        <v>145</v>
-      </c>
-      <c r="C8" t="s">
-        <v>183</v>
-      </c>
-      <c r="D8" t="s">
-        <v>151</v>
-      </c>
-      <c r="E8" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>147</v>
-      </c>
-      <c r="B9" s="14" t="s">
-        <v>144</v>
-      </c>
-      <c r="C9" t="s">
-        <v>184</v>
-      </c>
-      <c r="D9" t="s">
-        <v>152</v>
-      </c>
-      <c r="E9" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>147</v>
-      </c>
-      <c r="B10" s="14" t="s">
-        <v>145</v>
-      </c>
-      <c r="C10" t="s">
-        <v>185</v>
-      </c>
-      <c r="D10" t="s">
-        <v>152</v>
-      </c>
-      <c r="E10" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>148</v>
-      </c>
-      <c r="B11" s="14" t="s">
-        <v>144</v>
-      </c>
-      <c r="C11" t="s">
-        <v>186</v>
-      </c>
-      <c r="D11" t="s">
-        <v>153</v>
-      </c>
-      <c r="E11" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>148</v>
-      </c>
-      <c r="B12" s="14" t="s">
-        <v>145</v>
-      </c>
-      <c r="C12" t="s">
-        <v>187</v>
-      </c>
-      <c r="D12" t="s">
-        <v>153</v>
-      </c>
-      <c r="E12" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A13" s="14"/>
-      <c r="B13" s="14"/>
-      <c r="G13" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A14" s="4" t="s">
-        <v>159</v>
-      </c>
-      <c r="B14" s="25" t="s">
-        <v>154</v>
-      </c>
-      <c r="C14" s="4" t="s">
-        <v>162</v>
-      </c>
-      <c r="D14" s="11" t="s">
-        <v>149</v>
-      </c>
-      <c r="E14" s="11" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A15" s="4" t="s">
-        <v>159</v>
-      </c>
-      <c r="B15" s="25" t="s">
-        <v>155</v>
-      </c>
-      <c r="C15" s="4" t="s">
-        <v>163</v>
-      </c>
-      <c r="D15" s="11" t="s">
-        <v>150</v>
-      </c>
-      <c r="E15" s="11" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A16" s="4" t="s">
-        <v>159</v>
-      </c>
-      <c r="B16" s="25" t="s">
-        <v>156</v>
-      </c>
-      <c r="C16" s="4" t="s">
-        <v>164</v>
-      </c>
-      <c r="D16" s="11" t="s">
-        <v>151</v>
-      </c>
-      <c r="E16" s="11" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A17" s="4" t="s">
-        <v>159</v>
-      </c>
-      <c r="B17" s="25" t="s">
-        <v>157</v>
-      </c>
-      <c r="C17" s="4" t="s">
-        <v>165</v>
-      </c>
-      <c r="D17" s="11" t="s">
-        <v>152</v>
-      </c>
-      <c r="E17" s="11" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A18" s="4" t="s">
-        <v>159</v>
-      </c>
-      <c r="B18" s="25" t="s">
-        <v>158</v>
-      </c>
-      <c r="C18" s="4" t="s">
-        <v>166</v>
-      </c>
-      <c r="D18" s="11" t="s">
-        <v>153</v>
-      </c>
-      <c r="E18" s="11" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A19" s="26" t="s">
-        <v>160</v>
-      </c>
-      <c r="B19" s="27" t="s">
-        <v>154</v>
-      </c>
-      <c r="C19" s="26" t="s">
-        <v>167</v>
-      </c>
-      <c r="D19" s="11" t="s">
-        <v>149</v>
-      </c>
-      <c r="E19" s="11" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A20" s="26" t="s">
-        <v>160</v>
-      </c>
-      <c r="B20" s="27" t="s">
-        <v>155</v>
-      </c>
-      <c r="C20" s="26" t="s">
-        <v>168</v>
-      </c>
-      <c r="D20" s="11" t="s">
-        <v>150</v>
-      </c>
-      <c r="E20" s="11" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A21" s="26" t="s">
-        <v>160</v>
-      </c>
-      <c r="B21" s="27" t="s">
-        <v>156</v>
-      </c>
-      <c r="C21" s="26" t="s">
-        <v>169</v>
-      </c>
-      <c r="D21" s="11" t="s">
-        <v>151</v>
-      </c>
-      <c r="E21" s="11" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A22" s="26" t="s">
-        <v>160</v>
-      </c>
-      <c r="B22" s="27" t="s">
-        <v>157</v>
-      </c>
-      <c r="C22" s="26" t="s">
-        <v>170</v>
-      </c>
-      <c r="D22" s="11" t="s">
-        <v>152</v>
-      </c>
-      <c r="E22" s="11" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A23" s="26" t="s">
-        <v>160</v>
-      </c>
-      <c r="B23" s="27" t="s">
-        <v>158</v>
-      </c>
-      <c r="C23" s="26" t="s">
-        <v>171</v>
-      </c>
-      <c r="D23" s="11" t="s">
-        <v>153</v>
-      </c>
-      <c r="E23" s="11" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A24" s="28" t="s">
-        <v>161</v>
-      </c>
-      <c r="B24" s="29" t="s">
-        <v>154</v>
-      </c>
-      <c r="C24" s="28" t="s">
-        <v>172</v>
-      </c>
-      <c r="D24" s="11" t="s">
-        <v>149</v>
-      </c>
-      <c r="E24" s="11" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A25" s="28" t="s">
-        <v>161</v>
-      </c>
-      <c r="B25" s="29" t="s">
-        <v>155</v>
-      </c>
-      <c r="C25" s="28" t="s">
+      <c r="J27" s="2" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="28" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="F28" s="2" t="s">
+        <v>199</v>
+      </c>
+      <c r="G28" s="2" t="s">
+        <v>195</v>
+      </c>
+      <c r="H28" s="2" t="s">
         <v>173</v>
       </c>
-      <c r="D25" s="11" t="s">
-        <v>150</v>
-      </c>
-      <c r="E25" s="11" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A26" s="28" t="s">
-        <v>161</v>
-      </c>
-      <c r="B26" s="29" t="s">
-        <v>156</v>
-      </c>
-      <c r="C26" s="28" t="s">
+      <c r="I28" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="J28" s="2" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="29" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="F29" s="2" t="s">
+        <v>199</v>
+      </c>
+      <c r="G29" s="2" t="s">
+        <v>196</v>
+      </c>
+      <c r="H29" s="2" t="s">
         <v>174</v>
       </c>
-      <c r="D26" s="11" t="s">
-        <v>151</v>
-      </c>
-      <c r="E26" s="11" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A27" s="28" t="s">
-        <v>161</v>
-      </c>
-      <c r="B27" s="29" t="s">
-        <v>157</v>
-      </c>
-      <c r="C27" s="28" t="s">
+      <c r="I29" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="J29" s="2" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="30" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="F30" s="2" t="s">
+        <v>199</v>
+      </c>
+      <c r="G30" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="H30" s="2" t="s">
         <v>175</v>
       </c>
-      <c r="D27" s="11" t="s">
-        <v>152</v>
-      </c>
-      <c r="E27" s="11" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A28" s="28" t="s">
-        <v>161</v>
-      </c>
-      <c r="B28" s="29" t="s">
-        <v>158</v>
-      </c>
-      <c r="C28" s="28" t="s">
-        <v>176</v>
-      </c>
-      <c r="D28" s="11" t="s">
-        <v>153</v>
-      </c>
-      <c r="E28" s="11" t="s">
-        <v>158</v>
+      <c r="I30" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="J30" s="2" t="s">
+        <v>227</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0E083CA5-38D8-4145-BC52-D2EA97075D5E}">
+  <dimension ref="A1:B7"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="21.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.85546875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>152</v>
+      </c>
+      <c r="B1" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>153</v>
+      </c>
+      <c r="B2" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>154</v>
+      </c>
+      <c r="B3" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>155</v>
+      </c>
+      <c r="B4" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>156</v>
+      </c>
+      <c r="B5" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>157</v>
+      </c>
+      <c r="B6" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>158</v>
+      </c>
+      <c r="B7" t="s">
+        <v>165</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
igazából kész a packet
</commit_message>
<xml_diff>
--- a/Network/02.09 cimzes.xlsx
+++ b/Network/02.09 cimzes.xlsx
@@ -5,19 +5,20 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Felhasználó.GEP.000\Desktop\final-project-2025-26-main\final-project-2025-26-main\Network\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Github Repo\final-project-2025-26\Network\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A3791C5-ABE9-4D9A-BF12-10A502985E43}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{189B88D9-DF70-4666-B512-9AB60B60C246}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-105" windowWidth="29040" windowHeight="15840" activeTab="2" xr2:uid="{6F35F872-ABCC-42C2-B031-C1DE53122CDE}"/>
+    <workbookView xWindow="-28920" yWindow="-105" windowWidth="29040" windowHeight="15840" xr2:uid="{6F35F872-ABCC-42C2-B031-C1DE53122CDE}"/>
   </bookViews>
   <sheets>
     <sheet name="Telephelyek" sheetId="1" r:id="rId1"/>
     <sheet name="ISP Full Mesh" sheetId="4" r:id="rId2"/>
     <sheet name="ISP-telephelyek" sheetId="7" r:id="rId3"/>
-    <sheet name="OceanData" sheetId="8" r:id="rId4"/>
-    <sheet name="PAT" sheetId="9" r:id="rId5"/>
+    <sheet name="GRE over IPSec" sheetId="10" r:id="rId4"/>
+    <sheet name="OceanData" sheetId="8" r:id="rId5"/>
+    <sheet name="PAT" sheetId="9" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="315" uniqueCount="155">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="346" uniqueCount="178">
   <si>
     <t>Név</t>
   </si>
@@ -503,6 +504,75 @@
   </si>
   <si>
     <t>100.64.0.4/30</t>
+  </si>
+  <si>
+    <t>FactoryRouter</t>
+  </si>
+  <si>
+    <t>IrodaRouter</t>
+  </si>
+  <si>
+    <t>Tunnel0</t>
+  </si>
+  <si>
+    <t>172.100.0.1/30</t>
+  </si>
+  <si>
+    <t>172.100.0.2/30</t>
+  </si>
+  <si>
+    <t>172.100.0.5/30</t>
+  </si>
+  <si>
+    <t>172.100.0.6/30</t>
+  </si>
+  <si>
+    <t>172.100.0.9/30</t>
+  </si>
+  <si>
+    <t>172.100.0.10/30</t>
+  </si>
+  <si>
+    <t>172.100.0.13/30</t>
+  </si>
+  <si>
+    <t>172.100.0.14/30</t>
+  </si>
+  <si>
+    <t>172.100.0.17/30</t>
+  </si>
+  <si>
+    <t>172.100.0.18/30</t>
+  </si>
+  <si>
+    <t>2001:D88:100:1::1</t>
+  </si>
+  <si>
+    <t>2001:D88:100:1::2</t>
+  </si>
+  <si>
+    <t>Tunnel1</t>
+  </si>
+  <si>
+    <t>Tunnel2</t>
+  </si>
+  <si>
+    <t>Tunnel3</t>
+  </si>
+  <si>
+    <t>Tunnel4</t>
+  </si>
+  <si>
+    <t>Gyárüzem Firewall +  Szerver</t>
+  </si>
+  <si>
+    <t>192.168.200.0</t>
+  </si>
+  <si>
+    <t>192.168.200.1</t>
+  </si>
+  <si>
+    <t>255.255.255.252</t>
   </si>
 </sst>
 </file>
@@ -687,7 +757,9 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normál" xfId="0" builtinId="0"/>
@@ -1007,7 +1079,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B96E4ACA-B49F-4DB2-BCFB-280F26713B9B}">
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="43" bestFit="1" customWidth="1"/>
@@ -1080,49 +1152,64 @@
       <c r="E4" s="10"/>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" s="4" t="s">
+      <c r="A5" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>175</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>177</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>176</v>
+      </c>
+      <c r="E5" s="10"/>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="B6" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="C5" s="7" t="s">
+      <c r="C6" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="D5" s="7" t="s">
+      <c r="D6" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="E5" s="10"/>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" s="8" t="s">
+      <c r="E6" s="10"/>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="B6" s="8" t="s">
+      <c r="B7" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="C6" s="9" t="s">
+      <c r="C7" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="D6" s="8" t="s">
+      <c r="D7" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="E6" s="10"/>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7" s="6" t="s">
+      <c r="E7" s="10"/>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A8" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="B7" s="6" t="s">
+      <c r="B8" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="C7" s="6" t="s">
+      <c r="C8" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="D7" s="6" t="s">
+      <c r="D8" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="E7" s="10"/>
+      <c r="E8" s="10"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2029,6 +2116,119 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C53B8207-4E04-4A0B-B1B4-9436DF906978}">
+  <dimension ref="A1:G5"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="15.85546875" customWidth="1"/>
+    <col min="2" max="2" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="21.42578125" customWidth="1"/>
+    <col min="5" max="5" width="14.7109375" customWidth="1"/>
+    <col min="6" max="6" width="16.42578125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="16.28515625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>155</v>
+      </c>
+      <c r="B1" t="s">
+        <v>157</v>
+      </c>
+      <c r="C1" t="s">
+        <v>158</v>
+      </c>
+      <c r="D1" t="s">
+        <v>168</v>
+      </c>
+      <c r="E1" t="s">
+        <v>151</v>
+      </c>
+      <c r="F1" t="s">
+        <v>159</v>
+      </c>
+      <c r="G1" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>155</v>
+      </c>
+      <c r="B2" t="s">
+        <v>170</v>
+      </c>
+      <c r="C2" s="19" t="s">
+        <v>160</v>
+      </c>
+      <c r="D2" s="19"/>
+      <c r="E2" t="s">
+        <v>152</v>
+      </c>
+      <c r="F2" s="19" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>156</v>
+      </c>
+      <c r="B3" t="s">
+        <v>171</v>
+      </c>
+      <c r="C3" s="19" t="s">
+        <v>162</v>
+      </c>
+      <c r="D3" s="19"/>
+      <c r="E3" t="s">
+        <v>151</v>
+      </c>
+      <c r="F3" s="19" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>156</v>
+      </c>
+      <c r="B4" t="s">
+        <v>172</v>
+      </c>
+      <c r="C4" s="19" t="s">
+        <v>164</v>
+      </c>
+      <c r="D4" s="19"/>
+      <c r="E4" t="s">
+        <v>152</v>
+      </c>
+      <c r="F4" s="19" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>155</v>
+      </c>
+      <c r="B5" t="s">
+        <v>173</v>
+      </c>
+      <c r="C5" s="19" t="s">
+        <v>166</v>
+      </c>
+      <c r="D5" s="19"/>
+      <c r="E5" t="s">
+        <v>156</v>
+      </c>
+      <c r="F5" s="19" t="s">
+        <v>167</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2D271391-A8EE-41A4-AEE1-16B3367C6D79}">
   <dimension ref="A1:D6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2060,7 +2260,7 @@
       <c r="B2" t="s">
         <v>132</v>
       </c>
-      <c r="C2" s="19" t="s">
+      <c r="C2" t="s">
         <v>149</v>
       </c>
       <c r="D2" t="s">
@@ -2074,7 +2274,7 @@
       <c r="B3" t="s">
         <v>136</v>
       </c>
-      <c r="C3" s="19" t="s">
+      <c r="C3" t="s">
         <v>149</v>
       </c>
       <c r="D3" t="s">
@@ -2088,7 +2288,7 @@
       <c r="B4" t="s">
         <v>137</v>
       </c>
-      <c r="C4" s="19" t="s">
+      <c r="C4" t="s">
         <v>149</v>
       </c>
       <c r="D4" t="s">
@@ -2102,7 +2302,7 @@
       <c r="B5" t="s">
         <v>139</v>
       </c>
-      <c r="C5" s="19" t="s">
+      <c r="C5" t="s">
         <v>149</v>
       </c>
       <c r="D5" t="s">
@@ -2116,7 +2316,7 @@
       <c r="B6" t="s">
         <v>138</v>
       </c>
-      <c r="C6" s="19" t="s">
+      <c r="C6" t="s">
         <v>149</v>
       </c>
       <c r="D6" t="s">
@@ -2129,7 +2329,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7CF7C11D-B35F-4E63-B1DE-46E390154830}">
   <dimension ref="A2:A5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>

</xml_diff>

<commit_message>
Már csak a jelszavak, dokumentálás van
</commit_message>
<xml_diff>
--- a/Network/02.09 cimzes.xlsx
+++ b/Network/02.09 cimzes.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Github Repo\final-project-2025-26\Network\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{189B88D9-DF70-4666-B512-9AB60B60C246}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8FEAB69-03AF-4D5A-A087-2A9A2C07DC9C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-105" windowWidth="29040" windowHeight="15840" xr2:uid="{6F35F872-ABCC-42C2-B031-C1DE53122CDE}"/>
+    <workbookView xWindow="-28920" yWindow="-105" windowWidth="29040" windowHeight="15840" activeTab="4" xr2:uid="{6F35F872-ABCC-42C2-B031-C1DE53122CDE}"/>
   </bookViews>
   <sheets>
     <sheet name="Telephelyek" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="346" uniqueCount="178">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="350" uniqueCount="181">
   <si>
     <t>Név</t>
   </si>
@@ -573,6 +573,15 @@
   </si>
   <si>
     <t>255.255.255.252</t>
+  </si>
+  <si>
+    <t>SQL BKP</t>
+  </si>
+  <si>
+    <t>192.168.20.9</t>
+  </si>
+  <si>
+    <t>100.64.0.23</t>
   </si>
 </sst>
 </file>
@@ -2230,7 +2239,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2D271391-A8EE-41A4-AEE1-16B3367C6D79}">
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:D7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="21.7109375" bestFit="1" customWidth="1"/>
@@ -2321,6 +2330,20 @@
       </c>
       <c r="D6" t="s">
         <v>144</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>178</v>
+      </c>
+      <c r="B7" t="s">
+        <v>179</v>
+      </c>
+      <c r="C7" t="s">
+        <v>149</v>
+      </c>
+      <c r="D7" t="s">
+        <v>180</v>
       </c>
     </row>
   </sheetData>

</xml_diff>